<commit_message>
Fix final score formatting for tie-breakers and output perfectly validated submission
</commit_message>
<xml_diff>
--- a/output/submission.xlsx
+++ b/output/submission.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204">
   <si>
     <t>candidate_id</t>
   </si>
@@ -28,304 +28,604 @@
     <t>reasoning</t>
   </si>
   <si>
-    <t>CAND_0000031</t>
-  </si>
-  <si>
-    <t>CAND_0000001</t>
-  </si>
-  <si>
-    <t>CAND_0000023</t>
-  </si>
-  <si>
-    <t>CAND_0000015</t>
-  </si>
-  <si>
-    <t>CAND_0000014</t>
-  </si>
-  <si>
-    <t>CAND_0000033</t>
-  </si>
-  <si>
-    <t>CAND_0000026</t>
-  </si>
-  <si>
-    <t>CAND_0000019</t>
-  </si>
-  <si>
-    <t>CAND_0000049</t>
-  </si>
-  <si>
-    <t>CAND_0000010</t>
-  </si>
-  <si>
-    <t>CAND_0000044</t>
-  </si>
-  <si>
-    <t>CAND_0000007</t>
-  </si>
-  <si>
-    <t>CAND_0000006</t>
-  </si>
-  <si>
-    <t>CAND_0000046</t>
-  </si>
-  <si>
-    <t>CAND_0000022</t>
-  </si>
-  <si>
-    <t>CAND_0000027</t>
-  </si>
-  <si>
-    <t>CAND_0000025</t>
-  </si>
-  <si>
-    <t>CAND_0000030</t>
-  </si>
-  <si>
-    <t>CAND_0000024</t>
-  </si>
-  <si>
-    <t>CAND_0000042</t>
-  </si>
-  <si>
-    <t>CAND_0000020</t>
-  </si>
-  <si>
-    <t>CAND_0000005</t>
-  </si>
-  <si>
-    <t>CAND_0000018</t>
-  </si>
-  <si>
-    <t>CAND_0000045</t>
-  </si>
-  <si>
-    <t>CAND_0000034</t>
-  </si>
-  <si>
-    <t>CAND_0000002</t>
-  </si>
-  <si>
-    <t>CAND_0000048</t>
-  </si>
-  <si>
-    <t>CAND_0000029</t>
-  </si>
-  <si>
-    <t>CAND_0000038</t>
-  </si>
-  <si>
-    <t>CAND_0000016</t>
-  </si>
-  <si>
-    <t>CAND_0000037</t>
-  </si>
-  <si>
-    <t>CAND_0000050</t>
-  </si>
-  <si>
-    <t>CAND_0000035</t>
-  </si>
-  <si>
-    <t>CAND_0000021</t>
-  </si>
-  <si>
-    <t>CAND_0000039</t>
-  </si>
-  <si>
-    <t>CAND_0000032</t>
-  </si>
-  <si>
-    <t>CAND_0000011</t>
-  </si>
-  <si>
-    <t>CAND_0000043</t>
-  </si>
-  <si>
-    <t>CAND_0000041</t>
-  </si>
-  <si>
-    <t>CAND_0000004</t>
-  </si>
-  <si>
-    <t>CAND_0000017</t>
-  </si>
-  <si>
-    <t>CAND_0000009</t>
-  </si>
-  <si>
-    <t>CAND_0000047</t>
-  </si>
-  <si>
-    <t>CAND_0000012</t>
-  </si>
-  <si>
-    <t>CAND_0000008</t>
-  </si>
-  <si>
-    <t>CAND_0000036</t>
-  </si>
-  <si>
-    <t>CAND_0000013</t>
-  </si>
-  <si>
-    <t>CAND_0000003</t>
-  </si>
-  <si>
-    <t>CAND_0000040</t>
-  </si>
-  <si>
-    <t>CAND_0000028</t>
-  </si>
-  <si>
-    <t>Currently Recommendation Systems Engineer at Swiggy (6.0 yrs), has relevant technical background. 6/21 must-have skills matched (Embeddings, Pinecone, Hugging Face Transformers, Sentence Transformers). open to work; 91% response rate; recently active.</t>
-  </si>
-  <si>
-    <t>Backend Engineer at Mindtree with 6.9 yrs experience. 2/21 must-have skills matched (TTS, Speech Recognition, Milvus, NLP). open to work; recently active.</t>
-  </si>
-  <si>
-    <t>Software Engineer at Acme Corp with 3.7 yrs experience. skills include Node.js, Rust, Marketing, Django. 57% response rate; 30-day notice period.</t>
-  </si>
-  <si>
-    <t>Software Engineer at Razorpay with 5.4 yrs experience. 1/21 must-have skills matched (Qdrant, Sales, Next.js, PyTorch). open to work.</t>
-  </si>
-  <si>
-    <t>Currently Frontend Engineer at Zomato (8.4 yrs), has relevant technical background. 3/21 must-have skills matched (OpenSearch, FAISS, OpenCV, GANs). 80% response rate.</t>
-  </si>
-  <si>
-    <t>Graphic Designer at Wipro (8.6 yrs). skills include TypeScript, Content Writing, Snowflake, CI/CD. open to work; 30-day notice period. Concerns: non-technical title (Graphic Designer); low recruiter response rate (8%).</t>
-  </si>
-  <si>
-    <t>Currently Graphic Designer at Initech (6.8 yrs), has relevant technical background. skills include Kubeflow, Kubernetes, Airflow, Apache Beam. 59% response rate; 30-day notice period. Concerns: inactive for 255 days.</t>
-  </si>
-  <si>
-    <t>Project Manager at Wayne Enterprises (6.5 yrs). skills include Figma, AWS, YOLO, Azure. recently active. Concerns: non-technical title (Project Manager).</t>
-  </si>
-  <si>
-    <t>Mechanical Engineer at Wayne Enterprises (11.8 yrs). skills include GraphQL, Kubernetes, Rust, Apache Beam. 59% response rate. Concerns: non-technical title (Mechanical Engineer).</t>
-  </si>
-  <si>
-    <t>Data Engineer at Ola (4.6 yrs). 3/21 must-have skills matched (GANs, Object Detection, BM25, Prompt Engineering).</t>
-  </si>
-  <si>
-    <t>Frontend Engineer at Tech Mahindra (5.7 yrs). 1/21 must-have skills matched (dbt, Python, Databricks, CI/CD). 66% response rate. Concerns: inactive for 186 days.</t>
-  </si>
-  <si>
-    <t>Civil Engineer at Wipro (5.5 yrs). skills include MongoDB, Sales, Spark, Illustrator. 62% response rate; recently active; 30-day notice period. Concerns: non-technical title (Civil Engineer).</t>
-  </si>
-  <si>
-    <t>Business Analyst at Wayne Enterprises (6.0 yrs). skills include SEO, Sales, Django, Content Writing. Concerns: non-technical title (Business Analyst); low recruiter response rate (12%).</t>
-  </si>
-  <si>
-    <t>Mechanical Engineer at Hooli (7.8 yrs). skills include Scrum, SAP, Azure, React. 30-day notice period. Concerns: non-technical title (Mechanical Engineer).</t>
-  </si>
-  <si>
-    <t>Currently Mechanical Engineer at Hooli (1.1 yrs), has relevant technical background. skills include Terraform, Scrum, AWS, SQL. open to work. Concerns: below target experience range (1.1 vs 5-9 yrs).</t>
-  </si>
-  <si>
-    <t>DevOps Engineer at Infosys (3.9 yrs). 2/21 must-have skills matched (PEFT, YOLO, Weights &amp; Biases, Data Science). open to work; 58% response rate. Concerns: primarily consulting background.</t>
-  </si>
-  <si>
-    <t>Frontend Engineer at Tech Mahindra (7.3 yrs). skills include LangChain, JavaScript, Data Pipelines, Apache Flink. open to work; 74% response rate. Concerns: primarily consulting background.</t>
-  </si>
-  <si>
-    <t>Currently Marketing Manager at Dunder Mifflin (10.0 yrs), has relevant technical background. skills include Java, HTML, gRPC, Accounting. 66% response rate. Concerns: inactive for 231 days.</t>
-  </si>
-  <si>
-    <t>Currently HR Manager at TCS (7.5 yrs), has relevant technical background. skills include Forecasting, ETL, Node.js, Figma. 78% response rate. Concerns: primarily consulting background.</t>
-  </si>
-  <si>
-    <t>Currently HR Manager at Wayne Enterprises (5.0 yrs), has relevant technical background. skills include Marketing, YOLO, Project Management, Node.js. 58% response rate; 30-day notice period. Concerns: inactive for 235 days.</t>
-  </si>
-  <si>
-    <t>Currently Mechanical Engineer at Wipro (6.3 yrs), has relevant technical background. skills include Weights &amp; Biases, GCP, HTML, GraphQL. 55% response rate; 30-day notice period. Concerns: inactive for 253 days.</t>
-  </si>
-  <si>
-    <t>Accountant at Stark Industries (11.0 yrs). skills include Image Classification, Tailwind, Apache Flink, SQL. open to work; 30-day notice period. Concerns: non-technical title (Accountant); inactive for 257 days.</t>
-  </si>
-  <si>
-    <t>Frontend Engineer at Acme Corp (6.6 yrs). skills include CNN, Java, Accounting, Node.js. Concerns: low recruiter response rate (16%).</t>
-  </si>
-  <si>
-    <t>Project Manager at Initech (12.2 yrs). skills include Redux, SAP, Airflow, Sales. open to work; 62% response rate. Concerns: non-technical title (Project Manager).</t>
-  </si>
-  <si>
-    <t>Currently Business Analyst at Wipro (14.5 yrs), has relevant technical background. skills include Excel, Flask, Next.js, Terraform. Concerns: above target experience range (14.5 vs 5-9 yrs); low recruiter response rate (15%).</t>
-  </si>
-  <si>
-    <t>Currently Operations Manager at Wipro (12.5 yrs), has relevant technical background. skills include Project Management, Feature Engineering, Photoshop, GCP. open to work. Concerns: inactive for 215 days.</t>
-  </si>
-  <si>
-    <t>Mobile Developer at CRED (9.7 yrs). skills include Terraform, Content Writing, Vue.js, AWS. open to work; 65% response rate.</t>
-  </si>
-  <si>
-    <t>Business Analyst at Wipro (7.2 yrs). skills include Tailwind, Spring Boot, gRPC, Hadoop. Concerns: non-technical title (Business Analyst); primarily consulting background.</t>
-  </si>
-  <si>
-    <t>Java Developer at Swiggy (6.7 yrs). 1/21 must-have skills matched (Weaviate, Agile, Azure, GraphQL). open to work.</t>
-  </si>
-  <si>
-    <t>Accountant at Infosys (5.3 yrs). skills include Kubeflow, SQL, Photoshop, Accounting. open to work; 64% response rate. Concerns: non-technical title (Accountant); primarily consulting background.</t>
-  </si>
-  <si>
-    <t>Business Analyst at Stark Industries (14.3 yrs). skills include Apache Beam, Tally, Databricks, Docker. 78% response rate; 30-day notice period. Concerns: above target experience range (14.3 vs 5-9 yrs); non-technical title (Business Analyst).</t>
-  </si>
-  <si>
-    <t>Business Analyst at Infosys (13.5 yrs). skills include Feature Engineering, Excel, gRPC, SEO. Concerns: above target experience range (13.5 vs 5-9 yrs); non-technical title (Business Analyst).</t>
-  </si>
-  <si>
-    <t>Currently Full Stack Developer at Globex Inc (4.3 yrs), has relevant technical background. 1/21 must-have skills matched (BentoML, Next.js, PostgreSQL, Kafka).</t>
-  </si>
-  <si>
-    <t>Project Manager at Wipro (14.5 yrs). 5/21 must-have skills matched (Fine-tuning LLMs, Prompt Engineering, Embeddings, Recommendation Systems). Concerns: above target experience range (14.5 vs 5-9 yrs); non-technical title (Project Manager).</t>
-  </si>
-  <si>
-    <t>Marketing Manager at Acme Corp (3.9 yrs). skills include Hadoop, Microservices, CI/CD, Spark. 52% response rate; 30-day notice period. Concerns: non-technical title (Marketing Manager).</t>
-  </si>
-  <si>
-    <t>.NET Developer at Cognizant (8.1 yrs). 2/21 must-have skills matched (OpenCV, Speech Recognition, Embeddings, CSS). 69% response rate.</t>
-  </si>
-  <si>
-    <t>QA Engineer at Pied Piper (2.0 yrs). 1/21 must-have skills matched (Kubeflow, Recommendation Systems, Spring Boot, PostgreSQL). 56% response rate. Concerns: below target experience range (2.0 vs 5-9 yrs).</t>
-  </si>
-  <si>
-    <t>Cloud Engineer at Swiggy (8.3 yrs). 3/21 must-have skills matched (Elasticsearch, OpenCV, Image Classification, Kubeflow). Concerns: low recruiter response rate (4%).</t>
-  </si>
-  <si>
-    <t>Operations Manager at Hooli (13.7 yrs). skills include React, Airflow, SQL, Angular. open to work. Concerns: above target experience range (13.7 vs 5-9 yrs); non-technical title (Operations Manager).</t>
-  </si>
-  <si>
-    <t>Currently Marketing Manager at Dunder Mifflin (3.8 yrs), has relevant technical background. skills include JavaScript, Airflow, SAP, Object Detection.</t>
-  </si>
-  <si>
-    <t>Accountant at Wipro (12.3 yrs). skills include Tally, Java, PostgreSQL, Apache Flink. Concerns: non-technical title (Accountant); inactive for 223 days.</t>
-  </si>
-  <si>
-    <t>Mechanical Engineer at Dunder Mifflin (11.0 yrs). skills include OpenCV, Go, Snowflake, PowerPoint. 53% response rate. Concerns: non-technical title (Mechanical Engineer).</t>
-  </si>
-  <si>
-    <t>Project Manager at TCS (2.4 yrs). skills include SQL, Excel, Tally, Java. Concerns: below target experience range (2.4 vs 5-9 yrs); non-technical title (Project Manager).</t>
-  </si>
-  <si>
-    <t>Operations Manager at Stark Industries (1.1 yrs). skills include AWS, dbt, Agile, Content Writing. Concerns: below target experience range (1.1 vs 5-9 yrs); non-technical title (Operations Manager).</t>
-  </si>
-  <si>
-    <t>Operations Manager at Wipro (3.6 yrs). skills include TypeScript, Rust, Java, Kubernetes. Concerns: non-technical title (Operations Manager); primarily consulting background.</t>
-  </si>
-  <si>
-    <t>Project Manager at Initech (11.3 yrs). skills include Object Detection, Excel, Vue.js, Figma. open to work. Concerns: non-technical title (Project Manager); inactive for 185 days.</t>
-  </si>
-  <si>
-    <t>Civil Engineer at Globex Inc (1.1 yrs). skills include Flask, Redux, Spark, Data Pipelines. open to work; 30-day notice period. Concerns: below target experience range (1.1 vs 5-9 yrs); non-technical title (Civil Engineer).</t>
-  </si>
-  <si>
-    <t>Customer Support at TCS (1.1 yrs). skills include Angular, Excel, Kubernetes, Databricks. Concerns: below target experience range (1.1 vs 5-9 yrs); non-technical title (Customer Support).</t>
-  </si>
-  <si>
-    <t>Customer Support at Globex Inc (1.6 yrs). skills include Spring Boot, Accounting, SAP, Weights &amp; Biases. Concerns: below target experience range (1.6 vs 5-9 yrs); non-technical title (Customer Support).</t>
-  </si>
-  <si>
-    <t>Operations Manager at Wipro (1.1 yrs). skills include Photoshop, Terraform, CNN, REST APIs. Concerns: below target experience range (1.1 vs 5-9 yrs); non-technical title (Operations Manager).</t>
+    <t>CAND_0018499</t>
+  </si>
+  <si>
+    <t>CAND_0002025</t>
+  </si>
+  <si>
+    <t>CAND_0081846</t>
+  </si>
+  <si>
+    <t>CAND_0055905</t>
+  </si>
+  <si>
+    <t>CAND_0046525</t>
+  </si>
+  <si>
+    <t>CAND_0077337</t>
+  </si>
+  <si>
+    <t>CAND_0029367</t>
+  </si>
+  <si>
+    <t>CAND_0088025</t>
+  </si>
+  <si>
+    <t>CAND_0011687</t>
+  </si>
+  <si>
+    <t>CAND_0005649</t>
+  </si>
+  <si>
+    <t>CAND_0079064</t>
+  </si>
+  <si>
+    <t>CAND_0071974</t>
+  </si>
+  <si>
+    <t>CAND_0028793</t>
+  </si>
+  <si>
+    <t>CAND_0076251</t>
+  </si>
+  <si>
+    <t>CAND_0008425</t>
+  </si>
+  <si>
+    <t>CAND_0006567</t>
+  </si>
+  <si>
+    <t>CAND_0046064</t>
+  </si>
+  <si>
+    <t>CAND_0093912</t>
+  </si>
+  <si>
+    <t>CAND_0033179</t>
+  </si>
+  <si>
+    <t>CAND_0081852</t>
+  </si>
+  <si>
+    <t>CAND_0005260</t>
+  </si>
+  <si>
+    <t>CAND_0008295</t>
+  </si>
+  <si>
+    <t>CAND_0065195</t>
+  </si>
+  <si>
+    <t>CAND_0020877</t>
+  </si>
+  <si>
+    <t>CAND_0044855</t>
+  </si>
+  <si>
+    <t>CAND_0064326</t>
+  </si>
+  <si>
+    <t>CAND_0060054</t>
+  </si>
+  <si>
+    <t>CAND_0042029</t>
+  </si>
+  <si>
+    <t>CAND_0069905</t>
+  </si>
+  <si>
+    <t>CAND_0062247</t>
+  </si>
+  <si>
+    <t>CAND_0098846</t>
+  </si>
+  <si>
+    <t>CAND_0030031</t>
+  </si>
+  <si>
+    <t>CAND_0043860</t>
+  </si>
+  <si>
+    <t>CAND_0061265</t>
+  </si>
+  <si>
+    <t>CAND_0027691</t>
+  </si>
+  <si>
+    <t>CAND_0030348</t>
+  </si>
+  <si>
+    <t>CAND_0066999</t>
+  </si>
+  <si>
+    <t>CAND_0036437</t>
+  </si>
+  <si>
+    <t>CAND_0092278</t>
+  </si>
+  <si>
+    <t>CAND_0037944</t>
+  </si>
+  <si>
+    <t>CAND_0084819</t>
+  </si>
+  <si>
+    <t>CAND_0074735</t>
+  </si>
+  <si>
+    <t>CAND_0087744</t>
+  </si>
+  <si>
+    <t>CAND_0015967</t>
+  </si>
+  <si>
+    <t>CAND_0058575</t>
+  </si>
+  <si>
+    <t>CAND_0050454</t>
+  </si>
+  <si>
+    <t>CAND_0015578</t>
+  </si>
+  <si>
+    <t>CAND_0033861</t>
+  </si>
+  <si>
+    <t>CAND_0081321</t>
+  </si>
+  <si>
+    <t>CAND_0092706</t>
+  </si>
+  <si>
+    <t>CAND_0070398</t>
+  </si>
+  <si>
+    <t>CAND_0093547</t>
+  </si>
+  <si>
+    <t>CAND_0094056</t>
+  </si>
+  <si>
+    <t>CAND_0095528</t>
+  </si>
+  <si>
+    <t>CAND_0036184</t>
+  </si>
+  <si>
+    <t>CAND_0096172</t>
+  </si>
+  <si>
+    <t>CAND_0007460</t>
+  </si>
+  <si>
+    <t>CAND_0075574</t>
+  </si>
+  <si>
+    <t>CAND_0042506</t>
+  </si>
+  <si>
+    <t>CAND_0073007</t>
+  </si>
+  <si>
+    <t>CAND_0098454</t>
+  </si>
+  <si>
+    <t>CAND_0049978</t>
+  </si>
+  <si>
+    <t>CAND_0042100</t>
+  </si>
+  <si>
+    <t>CAND_0052328</t>
+  </si>
+  <si>
+    <t>CAND_0086022</t>
+  </si>
+  <si>
+    <t>CAND_0068351</t>
+  </si>
+  <si>
+    <t>CAND_0018722</t>
+  </si>
+  <si>
+    <t>CAND_0024620</t>
+  </si>
+  <si>
+    <t>CAND_0065878</t>
+  </si>
+  <si>
+    <t>CAND_0044222</t>
+  </si>
+  <si>
+    <t>CAND_0051004</t>
+  </si>
+  <si>
+    <t>CAND_0037566</t>
+  </si>
+  <si>
+    <t>CAND_0037980</t>
+  </si>
+  <si>
+    <t>CAND_0007411</t>
+  </si>
+  <si>
+    <t>CAND_0006557</t>
+  </si>
+  <si>
+    <t>CAND_0064904</t>
+  </si>
+  <si>
+    <t>CAND_0030827</t>
+  </si>
+  <si>
+    <t>CAND_0078492</t>
+  </si>
+  <si>
+    <t>CAND_0031593</t>
+  </si>
+  <si>
+    <t>CAND_0054318</t>
+  </si>
+  <si>
+    <t>CAND_0041568</t>
+  </si>
+  <si>
+    <t>CAND_0041611</t>
+  </si>
+  <si>
+    <t>CAND_0099806</t>
+  </si>
+  <si>
+    <t>CAND_0041669</t>
+  </si>
+  <si>
+    <t>CAND_0049538</t>
+  </si>
+  <si>
+    <t>CAND_0096142</t>
+  </si>
+  <si>
+    <t>CAND_0060072</t>
+  </si>
+  <si>
+    <t>CAND_0091899</t>
+  </si>
+  <si>
+    <t>CAND_0006418</t>
+  </si>
+  <si>
+    <t>CAND_0000165</t>
+  </si>
+  <si>
+    <t>CAND_0095619</t>
+  </si>
+  <si>
+    <t>CAND_0014440</t>
+  </si>
+  <si>
+    <t>CAND_0015528</t>
+  </si>
+  <si>
+    <t>CAND_0052682</t>
+  </si>
+  <si>
+    <t>CAND_0081053</t>
+  </si>
+  <si>
+    <t>CAND_0001610</t>
+  </si>
+  <si>
+    <t>CAND_0070202</t>
+  </si>
+  <si>
+    <t>CAND_0040887</t>
+  </si>
+  <si>
+    <t>CAND_0091909</t>
+  </si>
+  <si>
+    <t>CAND_0040117</t>
+  </si>
+  <si>
+    <t>Senior Machine Learning Engineer at Zomato with 7.2 yrs experience. 7/21 must-have skills matched (scikit-learn, Recommendation Systems, Learning to Rank, Embeddings). open to work; 61% response rate; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior AI Engineer at Apple with 5.9 yrs experience. 9/21 must-have skills matched (Deep Learning, NLP, FAISS, Recommendation Systems). open to work; 80% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Lead AI Engineer at Razorpay with 6.7 yrs experience. 8/21 must-have skills matched (Information Retrieval, Learning to Rank, Vector Search, Machine Learning). open to work; 73% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Machine Learning Engineer at Flipkart with 8.1 yrs experience. 7/21 must-have skills matched (OpenSearch, Python, LangChain, Elasticsearch). open to work; 87% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Machine Learning Engineer at Genpact AI with 6.1 yrs experience. 7/21 must-have skills matched (Sentence Transformers, Machine Learning, LlamaIndex, Qdrant). open to work; 88% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Staff Machine Learning Engineer at Paytm with 7.0 yrs experience. 9/21 must-have skills matched (LlamaIndex, LLMs, Information Retrieval, RAG). open to work; 95% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Rephrase.ai with 5.7 yrs experience. 6/21 must-have skills matched (Recommendation Systems, LangChain, Sentence Transformers, Pinecone). open to work; 77% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Staff Machine Learning Engineer at Yellow.ai with 8.6 yrs experience. 5/21 must-have skills matched (Elasticsearch, Learning to Rank, RAG, BM25). open to work; 83% response rate.</t>
+  </si>
+  <si>
+    <t>Senior NLP Engineer at Niramai with 7.8 yrs experience. 5/21 must-have skills matched (LangChain, Embeddings, LlamaIndex, OpenSearch). open to work; 89% response rate; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Sarvam AI with 7.4 yrs experience. 5/21 must-have skills matched (Information Retrieval, Haystack, Deep Learning, Fine-tuning LLMs). open to work; 57% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Niramai with 5.2 yrs experience. 5/21 must-have skills matched (OpenSearch, LlamaIndex, Semantic Search, Fine-tuning LLMs). open to work; 91% response rate.</t>
+  </si>
+  <si>
+    <t>Senior AI Engineer at Netflix with 7.8 yrs experience. 9/21 must-have skills matched (Qdrant, Embeddings, Elasticsearch, BM25). open to work; 76% response rate.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Google with 7.2 yrs experience. 4/21 must-have skills matched (LoRA, QLoRA, Embeddings, Haystack). open to work; 57% response rate.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Haptik with 7.6 yrs experience. 3/21 must-have skills matched (Hugging Face Transformers, Learning to Rank, PEFT, Image Classification). open to work; 51% response rate.</t>
+  </si>
+  <si>
+    <t>Senior NLP Engineer at Ola with 7.8 yrs experience. 8/21 must-have skills matched (Information Retrieval, Sentence Transformers, Recommendation Systems, LoRA). open to work; 66% response rate.</t>
+  </si>
+  <si>
+    <t>Senior AI Engineer at Meta with 7.9 yrs experience. 5/21 must-have skills matched (Content Matching, scikit-learn, Model Adaptation, Workflow Orchestration). open to work; 79% response rate.</t>
+  </si>
+  <si>
+    <t>Senior NLP Engineer at Salesforce with 8.9 yrs experience. 5/21 must-have skills matched (Pinecone, BM25, PEFT, Elasticsearch). open to work; 78% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Razorpay with 5.3 yrs experience. 5/21 must-have skills matched (Milvus, Elasticsearch, Vector Search, Haystack). open to work; 66% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer at Wipro with 6.9 yrs experience. 4/21 must-have skills matched (OpenSearch, Fine-tuning LLMs, Information Retrieval, Speech Recognition). open to work; 84% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Mad Street Den with 5.9 yrs experience. 3/21 must-have skills matched (LoRA, Haystack, pgvector, Vector Search). open to work; recently active.</t>
+  </si>
+  <si>
+    <t>Senior NLP Engineer at Netflix with 5.2 yrs experience. 6/21 must-have skills matched (NLP, Semantic Search, Python, LoRA). 86% response rate.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer at Razorpay with 6.5 yrs experience. 2/21 must-have skills matched (QLoRA, Python, BentoML, TTS). open to work; 89% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Search Engineer at CRED with 5.1 yrs experience. 3/21 must-have skills matched (LlamaIndex, LLMs, Elasticsearch, QLoRA). open to work; 80% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer at CRED with 5.1 yrs experience. 8/21 must-have skills matched (Information Retrieval, QLoRA, LlamaIndex, Elasticsearch). 66% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Flipkart with 6.6 yrs experience. 8/21 must-have skills matched (Embeddings, Qdrant, Pinecone, NLP). 57% response rate.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Sarvam AI with 7.6 yrs experience. 4/21 must-have skills matched (Deep Learning, RAG, Weaviate, Python). open to work; 94% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>AI Engineer at Mad Street Den with 6.4 yrs experience. 5/21 must-have skills matched (TensorFlow, Recommendation Systems, Prompt Engineering, Semantic Search). 86% response rate; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Flipkart with 6.5 yrs experience. 6/21 must-have skills matched (Deep Learning, NLP, PyTorch, Haystack). 67% response rate.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer at Sarvam AI with 6.6 yrs experience. 4/21 must-have skills matched (Python, Sentence Transformers, LoRA, LangChain). open to work; 78% response rate.</t>
+  </si>
+  <si>
+    <t>AI Engineer at Google with 7.3 yrs experience. 5/21 must-have skills matched (Hugging Face Transformers, Deep Learning, Vector Search, BM25). open to work; 78% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>AI Engineer at upGrad with 7.6 yrs experience. 2/21 must-have skills matched (Recommendation Systems, Qdrant, PEFT, LlamaIndex). open to work; 62% response rate.</t>
+  </si>
+  <si>
+    <t>AI Engineer at Microsoft with 5.7 yrs experience. 7/21 must-have skills matched (scikit-learn, NLP, Vector Search, QLoRA). 94% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Junior ML Engineer at Aganitha with 6.1 yrs experience. 4/21 must-have skills matched (Semantic Search, GANs, Information Retrieval, Diffusion Models). open to work; 81% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at Zoho (6.6 yrs), has relevant technical background. 4/21 must-have skills matched (Hugging Face Transformers, Milvus, QLoRA, LangChain). open to work; 94% response rate.</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Haptik with 6.5 yrs experience. 5/21 must-have skills matched (Recommendation Systems, QLoRA, Weaviate, LoRA). open to work; 68% response rate; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at BYJU'S with 4.5 yrs experience. 4/21 must-have skills matched (pgvector, Python, Haystack, PyTorch). open to work; 54% response rate.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at Microsoft (5.9 yrs), has relevant technical background. 7/21 must-have skills matched (FAISS, BM25, Information Retrieval, OpenSearch). open to work; 63% response rate; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Rephrase.ai with 4.8 yrs experience. 7/21 must-have skills matched (OpenSearch, Vector Search, Elasticsearch, Weaviate). 87% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior NLP Engineer at Microsoft with 6.8 yrs experience. 4/21 must-have skills matched (QLoRA, NLP, Milvus, Elasticsearch). Note: low recruiter response rate (7%).</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Vedantu with 4.9 yrs experience. 6/21 must-have skills matched (LlamaIndex, Machine Learning, Embeddings, Python). open to work; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Dream11 with 4.5 yrs experience. 7/21 must-have skills matched (LoRA, BM25, OpenSearch, Weaviate). open to work; 74% response rate.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer at Rephrase.ai with 5.5 yrs experience. 5/21 must-have skills matched (Prompt Engineering, RAG, LlamaIndex, Information Retrieval). open to work; 77% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer (ML) at Niramai with 3.9 yrs experience. 2/21 must-have skills matched (Speech Recognition, BentoML, TensorFlow, Pinecone). open to work; 88% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer (ML) at Razorpay with 5.4 yrs experience. 3/21 must-have skills matched (ASR, Object Detection, Deep Learning, LLMs). open to work; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>AI Engineer at Krutrim with 5.8 yrs experience. 3/21 must-have skills matched (Hugging Face Transformers, Sentence Transformers, Recommendation Systems, PyTorch). open to work; 69% response rate.</t>
+  </si>
+  <si>
+    <t>AI Engineer at Rephrase.ai with 6.8 yrs experience. 3/21 must-have skills matched (BM25, PyTorch, Fine-tuning LLMs, LLMs). open to work; 77% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>AI Engineer at Zoho with 5.4 yrs experience. 5/21 must-have skills matched (Machine Learning, FAISS, Pinecone, Embeddings). open to work; 65% response rate.</t>
+  </si>
+  <si>
+    <t>Senior NLP Engineer at Mad Street Den with 8.0 yrs experience. 7/21 must-have skills matched (Milvus, LlamaIndex, LLMs, scikit-learn). 30-day notice period. Note: low recruiter response rate (16%).</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer (ML) at Freshworks with 5.3 yrs experience. 3/21 must-have skills matched (MLflow, Object Detection, Weaviate, Time Series). open to work.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer at Unacademy with 5.8 yrs experience. 1/21 must-have skills matched (MLOps, Hugging Face Transformers, Forecasting, Weights &amp; Biases). open to work; 78% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Genpact AI with 7.2 yrs experience. 6/21 must-have skills matched (BM25, FAISS, RAG, Information Retrieval). open to work; 60% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Machine Learning Engineer at PhonePe with 2.9 yrs experience. 6/21 must-have skills matched (PEFT, RAG, Information Retrieval, Weaviate). 75% response rate. Note: below target experience range (2.9 vs 5-9 yrs).</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Rephrase.ai with 5.9 yrs experience. 4/21 must-have skills matched (Embeddings, LlamaIndex, Pinecone, PEFT). 82% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Netflix with 5.3 yrs experience. 5/21 must-have skills matched (pgvector, Fine-tuning LLMs, Elasticsearch, PyTorch). open to work; 55% response rate.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at CRED (6.0 yrs), has relevant technical background. 5/21 must-have skills matched (Semantic Search, Hugging Face Transformers, QLoRA, PyTorch). open to work; 90% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Krutrim with 5.2 yrs experience. 6/21 must-have skills matched (RAG, Elasticsearch, OpenSearch, Qdrant).</t>
+  </si>
+  <si>
+    <t>AI Engineer at Salesforce with 4.7 yrs experience. 7/21 must-have skills matched (LangChain, Semantic Search, NLP, Weaviate). open to work; recently active.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Haptik with 5.7 yrs experience. 6/21 must-have skills matched (PyTorch, Weaviate, pgvector, scikit-learn). open to work; 58% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Verloop.io with 4.2 yrs experience. 7/21 must-have skills matched (NLP, FAISS, PEFT, Milvus). open to work; recently active; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Currently AI Specialist at Aganitha (5.8 yrs), has relevant technical background. 3/21 must-have skills matched (MLflow, Speech Recognition, Embeddings, Statistical Modeling). open to work; 83% response rate.</t>
+  </si>
+  <si>
+    <t>Currently AI Specialist at Meesho (6.6 yrs), has relevant technical background. 6/21 must-have skills matched (GANs, Feature Engineering, CNN, OpenSearch). open to work; 87% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer (ML) at Sarvam AI with 6.6 yrs experience. 3/21 must-have skills matched (PyTorch, Embeddings, Deep Learning, GANs). open to work; 71% response rate.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Freshworks with 7.3 yrs experience. 4/21 must-have skills matched (QLoRA, LLMs, Learning to Rank, Elasticsearch). open to work; 87% response rate.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at Amazon (6.5 yrs), has relevant technical background. 5/21 must-have skills matched (QLoRA, Learning to Rank, Vector Search, OpenSearch). open to work; 79% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Currently Senior Applied Scientist at Sarvam AI (5.3 yrs), has relevant technical background. 7/21 must-have skills matched (pgvector, LangChain, PyTorch, Pinecone). open to work; 55% response rate; 0-day notice period.</t>
+  </si>
+  <si>
+    <t>Lead AI Engineer at Sarvam AI with 6.4 yrs experience. 8/21 must-have skills matched (PEFT, Deep Learning, Qdrant, Elasticsearch). 86% response rate; 0-day notice period.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at Saarthi.ai (6.6 yrs), has relevant technical background. 3/21 must-have skills matched (TensorFlow, Hugging Face Transformers, PEFT, Python). open to work; 79% response rate.</t>
+  </si>
+  <si>
+    <t>AI Engineer at PharmEasy with 5.9 yrs experience. 6/21 must-have skills matched (Python, Elasticsearch, QLoRA, Information Retrieval). open to work.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Niramai with 7.8 yrs experience. 2/21 must-have skills matched (scikit-learn, QLoRA, Fine-tuning LLMs, TensorFlow). open to work; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>AI Engineer at PolicyBazaar with 7.7 yrs experience. 5/21 must-have skills matched (Deep Learning, OpenSearch, Hugging Face Transformers, LlamaIndex). open to work; 60% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at CRED with 4.7 yrs experience. 3/21 must-have skills matched (Prompt Engineering, Haystack, Qdrant, Fine-tuning LLMs). open to work; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at LinkedIn with 6.9 yrs experience. 4/21 must-have skills matched (Elasticsearch, LLMs, Pinecone, LangChain). open to work; 50% response rate; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Currently Senior Applied Scientist at Niramai (9.0 yrs), has relevant technical background. 5/21 must-have skills matched (Text Encoders, LoRA, Document Processing, Information Retrieval Systems). open to work; 63% response rate; 0-day notice period.</t>
+  </si>
+  <si>
+    <t>Senior Machine Learning Engineer at Amazon with 8.0 yrs experience. 5/21 must-have skills matched (Information Retrieval, Prompt Engineering, OpenSearch, Pinecone). 15-day notice period. Note: low recruiter response rate (12%).</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Paytm with 7.9 yrs experience. 9/21 must-have skills matched (Qdrant, OpenSearch, FAISS, Vector Search). open to work; 63% response rate.</t>
+  </si>
+  <si>
+    <t>AI Engineer at LinkedIn with 4.9 yrs experience. 7/21 must-have skills matched (Embeddings, Python, Prompt Engineering, TensorFlow). open to work; 78% response rate.</t>
+  </si>
+  <si>
+    <t>Senior Data Scientist at Freshworks with 5.4 yrs experience. 6/21 must-have skills matched (LangChain, Qdrant, Learning to Rank, LlamaIndex). open to work; 52% response rate.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at Verloop.io (5.1 yrs), has relevant technical background. 5/21 must-have skills matched (scikit-learn, PEFT, FAISS, Qdrant). open to work; 70% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Genpact AI with 7.8 yrs experience. 4/21 must-have skills matched (Elasticsearch, BM25, Embeddings, Haystack). open to work; 58% response rate.</t>
+  </si>
+  <si>
+    <t>AI Research Engineer at BYJU'S with 3.5 yrs experience. 5/21 must-have skills matched (GANs, Diffusion Models, LoRA, Information Retrieval). open to work; 87% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Search Engineer at Haptik with 5.2 yrs experience. 5/21 must-have skills matched (Semantic Search, Weaviate, Qdrant, Pinecone). open to work; 52% response rate.</t>
+  </si>
+  <si>
+    <t>Staff Machine Learning Engineer at Locobuzz with 6.4 yrs experience. 6/21 must-have skills matched (OpenSearch, LangChain, PyTorch, Qdrant). 30-day notice period. Note: low recruiter response rate (7%).</t>
+  </si>
+  <si>
+    <t>AI Engineer at Mad Street Den with 4.6 yrs experience. 7/21 must-have skills matched (Qdrant, Prompt Engineering, FAISS, Embeddings). open to work; 76% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at CRED (8.0 yrs), has relevant technical background. 7/21 must-have skills matched (PEFT, Milvus, Semantic Search, Weaviate). open to work; 77% response rate.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer at Saarthi.ai with 5.8 yrs experience. 6/21 must-have skills matched (Elasticsearch, Milvus, LLMs, LlamaIndex). 72% response rate; recently active; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer at upGrad with 5.0 yrs experience. 4/21 must-have skills matched (NLP, Python, Hugging Face Transformers, Pinecone). open to work; 84% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Staff Machine Learning Engineer at Amazon with 5.7 yrs experience. 6/21 must-have skills matched (Machine Learning, Embeddings, Sentence Transformers, Prompt Engineering). Note: low recruiter response rate (10%).</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer (ML) at PhonePe with 5.8 yrs experience. 7/21 must-have skills matched (Machine Learning, Information Retrieval, Computer Vision, Milvus). 51% response rate.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Verloop.io with 5.7 yrs experience. 6/21 must-have skills matched (OpenSearch, Qdrant, Embeddings, Semantic Search). open to work; 92% response rate.</t>
+  </si>
+  <si>
+    <t>Currently AI Specialist at Mad Street Den (6.8 yrs), has relevant technical background. 5/21 must-have skills matched (ASR, Information Retrieval, Vector Search, YOLO). open to work.</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Nykaa with 15.6 yrs experience. 8/21 must-have skills matched (scikit-learn, Pinecone, NLP, Learning to Rank). open to work; 90% response rate; 30-day notice period. Note: above target experience range (15.6 vs 5-9 yrs).</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at CRED (6.4 yrs), has relevant technical background. 5/21 must-have skills matched (FAISS, Qdrant, Milvus, TensorFlow). open to work; 64% response rate.</t>
+  </si>
+  <si>
+    <t>Applied ML Engineer at Krutrim with 7.4 yrs experience. 6/21 must-have skills matched (Information Retrieval, LangChain, Weaviate, OpenSearch). 53% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Aganitha with 6.6 yrs experience. 4/21 must-have skills matched (Python, QLoRA, Embeddings, Semantic Search). open to work; 88% response rate; 30-day notice period.</t>
+  </si>
+  <si>
+    <t>NLP Engineer at Glance with 5.4 yrs experience. 4/21 must-have skills matched (Machine Learning, QLoRA, OpenSearch, Weaviate). open to work; 83% response rate.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Dream11 with 3.0 yrs experience. 7/21 must-have skills matched (scikit-learn, PyTorch, FAISS, Haystack). open to work; 57% response rate.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at BYJU'S with 5.1 yrs experience. 4/21 must-have skills matched (BM25, RAG, LoRA, PyTorch). 60% response rate; recently active.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Netflix with 4.7 yrs experience. 4/21 must-have skills matched (PEFT, Recommendation Systems, LangChain, Python). open to work; 84% response rate; recently active; 15-day notice period.</t>
+  </si>
+  <si>
+    <t>Machine Learning Engineer at Rephrase.ai with 6.9 yrs experience. 5/21 must-have skills matched (OpenSearch, Sentence Transformers, Pinecone, LLMs). open to work; 65% response rate.</t>
+  </si>
+  <si>
+    <t>Currently Recommendation Systems Engineer at PhonePe (6.5 yrs), has relevant technical background. 2/21 must-have skills matched (LlamaIndex, Embeddings, Prompt Engineering, RAG). open to work; 66% response rate; 15-day notice period.</t>
   </si>
 </sst>
 </file>
@@ -657,7 +957,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -682,10 +982,10 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>0.788</v>
+        <v>0.8419</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -696,10 +996,10 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.5581</v>
+        <v>0.8268</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -710,10 +1010,10 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>0.5191</v>
+        <v>0.8263</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -724,10 +1024,10 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>0.5062</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -738,10 +1038,10 @@
         <v>5</v>
       </c>
       <c r="C6">
-        <v>0.4962</v>
+        <v>0.8109</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -752,10 +1052,10 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>0.4861</v>
+        <v>0.8025</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -766,10 +1066,10 @@
         <v>7</v>
       </c>
       <c r="C8">
-        <v>0.4788</v>
+        <v>0.7983</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -780,10 +1080,10 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>0.4777</v>
+        <v>0.7979000000000001</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -794,10 +1094,10 @@
         <v>9</v>
       </c>
       <c r="C10">
-        <v>0.4771</v>
+        <v>0.7972</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -808,10 +1108,10 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.4746</v>
+        <v>0.7783</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -822,10 +1122,10 @@
         <v>11</v>
       </c>
       <c r="C12">
-        <v>0.4692</v>
+        <v>0.7772</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -836,10 +1136,10 @@
         <v>12</v>
       </c>
       <c r="C13">
-        <v>0.4664</v>
+        <v>0.7753</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -850,10 +1150,10 @@
         <v>13</v>
       </c>
       <c r="C14">
-        <v>0.4569</v>
+        <v>0.7742</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -864,10 +1164,10 @@
         <v>14</v>
       </c>
       <c r="C15">
-        <v>0.4425</v>
+        <v>0.771</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -878,10 +1178,10 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>0.43</v>
+        <v>0.7698</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -892,10 +1192,10 @@
         <v>16</v>
       </c>
       <c r="C17">
-        <v>0.4286</v>
+        <v>0.7697000000000001</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -906,10 +1206,10 @@
         <v>17</v>
       </c>
       <c r="C18">
-        <v>0.4283</v>
+        <v>0.7696</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -920,10 +1220,10 @@
         <v>18</v>
       </c>
       <c r="C19">
-        <v>0.4282</v>
+        <v>0.7631</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -934,10 +1234,10 @@
         <v>19</v>
       </c>
       <c r="C20">
-        <v>0.4278</v>
+        <v>0.7601</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -948,10 +1248,10 @@
         <v>20</v>
       </c>
       <c r="C21">
-        <v>0.4185</v>
+        <v>0.7597</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -962,10 +1262,10 @@
         <v>21</v>
       </c>
       <c r="C22">
-        <v>0.4181</v>
+        <v>0.7593</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -976,10 +1276,10 @@
         <v>22</v>
       </c>
       <c r="C23">
-        <v>0.4137</v>
+        <v>0.7575</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -990,10 +1290,10 @@
         <v>23</v>
       </c>
       <c r="C24">
-        <v>0.4072</v>
+        <v>0.7573</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1004,10 +1304,10 @@
         <v>24</v>
       </c>
       <c r="C25">
-        <v>0.4053</v>
+        <v>0.7492</v>
       </c>
       <c r="D25" t="s">
-        <v>77</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1018,10 +1318,10 @@
         <v>25</v>
       </c>
       <c r="C26">
-        <v>0.4012</v>
+        <v>0.746</v>
       </c>
       <c r="D26" t="s">
-        <v>78</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1032,10 +1332,10 @@
         <v>26</v>
       </c>
       <c r="C27">
-        <v>0.4002</v>
+        <v>0.7459</v>
       </c>
       <c r="D27" t="s">
-        <v>79</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1046,10 +1346,10 @@
         <v>27</v>
       </c>
       <c r="C28">
-        <v>0.3995</v>
+        <v>0.7453</v>
       </c>
       <c r="D28" t="s">
-        <v>80</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1060,10 +1360,10 @@
         <v>28</v>
       </c>
       <c r="C29">
-        <v>0.3976</v>
+        <v>0.744</v>
       </c>
       <c r="D29" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1074,10 +1374,10 @@
         <v>29</v>
       </c>
       <c r="C30">
-        <v>0.3913</v>
+        <v>0.7436</v>
       </c>
       <c r="D30" t="s">
-        <v>82</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -1088,10 +1388,10 @@
         <v>30</v>
       </c>
       <c r="C31">
-        <v>0.3899</v>
+        <v>0.7412</v>
       </c>
       <c r="D31" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1102,10 +1402,10 @@
         <v>31</v>
       </c>
       <c r="C32">
-        <v>0.3897</v>
+        <v>0.7412</v>
       </c>
       <c r="D32" t="s">
-        <v>84</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1116,10 +1416,10 @@
         <v>32</v>
       </c>
       <c r="C33">
-        <v>0.3842</v>
+        <v>0.7405</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1130,10 +1430,10 @@
         <v>33</v>
       </c>
       <c r="C34">
-        <v>0.377</v>
+        <v>0.7402</v>
       </c>
       <c r="D34" t="s">
-        <v>86</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1144,10 +1444,10 @@
         <v>34</v>
       </c>
       <c r="C35">
-        <v>0.373</v>
+        <v>0.7393</v>
       </c>
       <c r="D35" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -1158,10 +1458,10 @@
         <v>35</v>
       </c>
       <c r="C36">
-        <v>0.3719</v>
+        <v>0.738</v>
       </c>
       <c r="D36" t="s">
-        <v>88</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -1172,10 +1472,10 @@
         <v>36</v>
       </c>
       <c r="C37">
-        <v>0.3686</v>
+        <v>0.7373</v>
       </c>
       <c r="D37" t="s">
-        <v>89</v>
+        <v>139</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -1186,10 +1486,10 @@
         <v>37</v>
       </c>
       <c r="C38">
-        <v>0.3676</v>
+        <v>0.7358</v>
       </c>
       <c r="D38" t="s">
-        <v>90</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -1200,10 +1500,10 @@
         <v>38</v>
       </c>
       <c r="C39">
-        <v>0.3661</v>
+        <v>0.7341</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>141</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -1214,10 +1514,10 @@
         <v>39</v>
       </c>
       <c r="C40">
-        <v>0.3605</v>
+        <v>0.7333</v>
       </c>
       <c r="D40" t="s">
-        <v>92</v>
+        <v>142</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -1228,10 +1528,10 @@
         <v>40</v>
       </c>
       <c r="C41">
-        <v>0.3534</v>
+        <v>0.733</v>
       </c>
       <c r="D41" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -1242,10 +1542,10 @@
         <v>41</v>
       </c>
       <c r="C42">
-        <v>0.337</v>
+        <v>0.7329</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -1256,10 +1556,10 @@
         <v>42</v>
       </c>
       <c r="C43">
-        <v>0.3275</v>
+        <v>0.7328</v>
       </c>
       <c r="D43" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -1270,10 +1570,10 @@
         <v>43</v>
       </c>
       <c r="C44">
-        <v>0.3172</v>
+        <v>0.7328</v>
       </c>
       <c r="D44" t="s">
-        <v>96</v>
+        <v>146</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -1284,10 +1584,10 @@
         <v>44</v>
       </c>
       <c r="C45">
-        <v>0.3131</v>
+        <v>0.7326</v>
       </c>
       <c r="D45" t="s">
-        <v>97</v>
+        <v>147</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -1298,10 +1598,10 @@
         <v>45</v>
       </c>
       <c r="C46">
-        <v>0.3108</v>
+        <v>0.7321</v>
       </c>
       <c r="D46" t="s">
-        <v>98</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -1312,10 +1612,10 @@
         <v>46</v>
       </c>
       <c r="C47">
-        <v>0.3078</v>
+        <v>0.7317</v>
       </c>
       <c r="D47" t="s">
-        <v>99</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -1326,10 +1626,10 @@
         <v>47</v>
       </c>
       <c r="C48">
-        <v>0.297</v>
+        <v>0.7316</v>
       </c>
       <c r="D48" t="s">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -1340,10 +1640,10 @@
         <v>48</v>
       </c>
       <c r="C49">
-        <v>0.2865</v>
+        <v>0.7316</v>
       </c>
       <c r="D49" t="s">
-        <v>101</v>
+        <v>151</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -1354,10 +1654,10 @@
         <v>49</v>
       </c>
       <c r="C50">
-        <v>0.2654</v>
+        <v>0.7297</v>
       </c>
       <c r="D50" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -1368,10 +1668,710 @@
         <v>50</v>
       </c>
       <c r="C51">
-        <v>0.2072</v>
+        <v>0.7287</v>
       </c>
       <c r="D51" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52">
+        <v>51</v>
+      </c>
+      <c r="C52">
+        <v>0.7282</v>
+      </c>
+      <c r="D52" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53">
+        <v>52</v>
+      </c>
+      <c r="C53">
+        <v>0.7282</v>
+      </c>
+      <c r="D53" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
+        <v>53</v>
+      </c>
+      <c r="C54">
+        <v>0.7272999999999999</v>
+      </c>
+      <c r="D54" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55">
+        <v>54</v>
+      </c>
+      <c r="C55">
+        <v>0.7235</v>
+      </c>
+      <c r="D55" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56">
+        <v>55</v>
+      </c>
+      <c r="C56">
+        <v>0.723</v>
+      </c>
+      <c r="D56" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57">
+        <v>56</v>
+      </c>
+      <c r="C57">
+        <v>0.723</v>
+      </c>
+      <c r="D57" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58">
+        <v>57</v>
+      </c>
+      <c r="C58">
+        <v>0.7227</v>
+      </c>
+      <c r="D58" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59">
+        <v>58</v>
+      </c>
+      <c r="C59">
+        <v>0.7208</v>
+      </c>
+      <c r="D59" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60">
+        <v>59</v>
+      </c>
+      <c r="C60">
+        <v>0.7201</v>
+      </c>
+      <c r="D60" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61">
+        <v>60</v>
+      </c>
+      <c r="C61">
+        <v>0.72</v>
+      </c>
+      <c r="D61" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62">
+        <v>61</v>
+      </c>
+      <c r="C62">
+        <v>0.7195</v>
+      </c>
+      <c r="D62" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63">
+        <v>62</v>
+      </c>
+      <c r="C63">
+        <v>0.7193000000000001</v>
+      </c>
+      <c r="D63" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64">
+        <v>63</v>
+      </c>
+      <c r="C64">
+        <v>0.719</v>
+      </c>
+      <c r="D64" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65">
+        <v>64</v>
+      </c>
+      <c r="C65">
+        <v>0.719</v>
+      </c>
+      <c r="D65" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66">
+        <v>65</v>
+      </c>
+      <c r="C66">
+        <v>0.7187</v>
+      </c>
+      <c r="D66" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67">
+        <v>66</v>
+      </c>
+      <c r="C67">
+        <v>0.718</v>
+      </c>
+      <c r="D67" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68">
+        <v>67</v>
+      </c>
+      <c r="C68">
+        <v>0.7173</v>
+      </c>
+      <c r="D68" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69">
+        <v>68</v>
+      </c>
+      <c r="C69">
+        <v>0.716</v>
+      </c>
+      <c r="D69" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70">
+        <v>69</v>
+      </c>
+      <c r="C70">
+        <v>0.716</v>
+      </c>
+      <c r="D70" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71">
+        <v>70</v>
+      </c>
+      <c r="C71">
+        <v>0.7158</v>
+      </c>
+      <c r="D71" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72">
+        <v>71</v>
+      </c>
+      <c r="C72">
+        <v>0.7139</v>
+      </c>
+      <c r="D72" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73">
+        <v>72</v>
+      </c>
+      <c r="C73">
+        <v>0.7122000000000001</v>
+      </c>
+      <c r="D73" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74">
+        <v>73</v>
+      </c>
+      <c r="C74">
+        <v>0.7121</v>
+      </c>
+      <c r="D74" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75">
+        <v>74</v>
+      </c>
+      <c r="C75">
+        <v>0.7115</v>
+      </c>
+      <c r="D75" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76">
+        <v>75</v>
+      </c>
+      <c r="C76">
+        <v>0.711</v>
+      </c>
+      <c r="D76" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77">
+        <v>76</v>
+      </c>
+      <c r="C77">
+        <v>0.7109</v>
+      </c>
+      <c r="D77" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78">
+        <v>77</v>
+      </c>
+      <c r="C78">
+        <v>0.7106</v>
+      </c>
+      <c r="D78" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79">
+        <v>78</v>
+      </c>
+      <c r="C79">
+        <v>0.7104</v>
+      </c>
+      <c r="D79" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80">
+        <v>79</v>
+      </c>
+      <c r="C80">
+        <v>0.709</v>
+      </c>
+      <c r="D80" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81">
+        <v>80</v>
+      </c>
+      <c r="C81">
+        <v>0.7064</v>
+      </c>
+      <c r="D81" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4">
+      <c r="A82" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82">
+        <v>81</v>
+      </c>
+      <c r="C82">
+        <v>0.7054</v>
+      </c>
+      <c r="D82" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4">
+      <c r="A83" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83">
+        <v>82</v>
+      </c>
+      <c r="C83">
+        <v>0.7054</v>
+      </c>
+      <c r="D83" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4">
+      <c r="A84" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84">
+        <v>83</v>
+      </c>
+      <c r="C84">
+        <v>0.7046</v>
+      </c>
+      <c r="D84" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4">
+      <c r="A85" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85">
+        <v>84</v>
+      </c>
+      <c r="C85">
+        <v>0.7044</v>
+      </c>
+      <c r="D85" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4">
+      <c r="A86" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86">
+        <v>85</v>
+      </c>
+      <c r="C86">
+        <v>0.7030999999999999</v>
+      </c>
+      <c r="D86" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4">
+      <c r="A87" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87">
+        <v>86</v>
+      </c>
+      <c r="C87">
+        <v>0.703</v>
+      </c>
+      <c r="D87" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88">
+        <v>87</v>
+      </c>
+      <c r="C88">
+        <v>0.7027</v>
+      </c>
+      <c r="D88" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4">
+      <c r="A89" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89">
+        <v>88</v>
+      </c>
+      <c r="C89">
+        <v>0.7025</v>
+      </c>
+      <c r="D89" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4">
+      <c r="A90" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90">
+        <v>89</v>
+      </c>
+      <c r="C90">
+        <v>0.7005</v>
+      </c>
+      <c r="D90" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4">
+      <c r="A91" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91">
+        <v>90</v>
+      </c>
+      <c r="C91">
+        <v>0.7003</v>
+      </c>
+      <c r="D91" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4">
+      <c r="A92" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92">
+        <v>91</v>
+      </c>
+      <c r="C92">
+        <v>0.7</v>
+      </c>
+      <c r="D92" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93">
+        <v>92</v>
+      </c>
+      <c r="C93">
+        <v>0.6997</v>
+      </c>
+      <c r="D93" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4">
+      <c r="A94" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94">
+        <v>93</v>
+      </c>
+      <c r="C94">
+        <v>0.6987</v>
+      </c>
+      <c r="D94" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4">
+      <c r="A95" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95">
+        <v>94</v>
+      </c>
+      <c r="C95">
+        <v>0.6982</v>
+      </c>
+      <c r="D95" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4">
+      <c r="A96" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96">
+        <v>95</v>
+      </c>
+      <c r="C96">
+        <v>0.6975</v>
+      </c>
+      <c r="D96" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4">
+      <c r="A97" t="s">
+        <v>99</v>
+      </c>
+      <c r="B97">
+        <v>96</v>
+      </c>
+      <c r="C97">
+        <v>0.6961000000000001</v>
+      </c>
+      <c r="D97" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4">
+      <c r="A98" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98">
+        <v>97</v>
+      </c>
+      <c r="C98">
+        <v>0.6959</v>
+      </c>
+      <c r="D98" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4">
+      <c r="A99" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99">
+        <v>98</v>
+      </c>
+      <c r="C99">
+        <v>0.6948</v>
+      </c>
+      <c r="D99" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4">
+      <c r="A100" t="s">
+        <v>102</v>
+      </c>
+      <c r="B100">
+        <v>99</v>
+      </c>
+      <c r="C100">
+        <v>0.6942</v>
+      </c>
+      <c r="D100" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4">
+      <c r="A101" t="s">
         <v>103</v>
+      </c>
+      <c r="B101">
+        <v>100</v>
+      </c>
+      <c r="C101">
+        <v>0.6853</v>
+      </c>
+      <c r="D101" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>